<commit_message>
Lock Faleth capsule slot 5 to Flint & Tinder Forest trucker
Lyle called F&T Forest the closest match; keep Quince/Gap/Blakely as Add-ons backups.
</commit_message>
<xml_diff>
--- a/Personal/Ideas/Faleth Wardrobe Capsule/Faleth Wardrobe Capsule.xlsx
+++ b/Personal/Ideas/Faleth Wardrobe Capsule/Faleth Wardrobe Capsule.xlsx
@@ -760,52 +760,52 @@
       </c>
     </row>
     <row r="6" ht="55" customHeight="1">
-      <c r="A6" s="6" t="n">
+      <c r="A6" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>Forest/olive denim or denim-look trucker / field</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>PRIMARY options ranked: (A) Quince Dark Forest waxed trucker $150 — or (B) Gap Surplus Green field $70 interim — or (C) Blakely olive denim-blend L in stock</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
-          <t>Dark Forest / Surplus Green / Olive</t>
-        </is>
-      </c>
-      <c r="E6" s="6" t="inlineStr">
-        <is>
-          <t>True forest denim OOS US. Quince: waxed canvas, dual flaps, metal shanks. Gap: herringbone field $70. Blakely: stretch denim blend, L live / XL OOS.</t>
-        </is>
-      </c>
-      <c r="F6" s="6" t="inlineStr">
-        <is>
-          <t>150 / 70 / 105</t>
-        </is>
-      </c>
-      <c r="G6" s="6" t="inlineStr">
-        <is>
-          <t>Start L; XL if heavy layers. Blakely: L only reliably.</t>
-        </is>
-      </c>
-      <c r="H6" s="6" t="inlineStr">
-        <is>
-          <t>LIVE options — pick after hardware decision</t>
-        </is>
-      </c>
-      <c r="I6" s="7" t="inlineStr">
-        <is>
-          <t>https://www.quince.com/men/mens-organic-cotton-wax-canvas-trucker-jacket?color=dark-forest-green</t>
-        </is>
-      </c>
-      <c r="J6" s="6" t="inlineStr">
-        <is>
-          <t>See Add-ons Slot5 for full ranked list + Buck Mason Soft Olive $298 + F&amp;T Forest $328</t>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>LOCKED: Flint &amp; Tinder Flannel-Lined Waxed Trucker (Huckberry) — Forest</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>Forest</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>Martexin 7oz waxed sailcloth, USA; antique-finish metal buttons; ONE button-flap chest pocket (not dual). Soft blanket lining.</t>
+        </is>
+      </c>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>328</t>
+        </is>
+      </c>
+      <c r="G6" s="8" t="inlineStr">
+        <is>
+          <t>Start XL if you usually L–XL and layer (brand runs trim); else L</t>
+        </is>
+      </c>
+      <c r="H6" s="8" t="inlineStr">
+        <is>
+          <t>LOCKED — Lyle pick 2026-09-05 (closest so far)</t>
+        </is>
+      </c>
+      <c r="I6" s="9" t="inlineStr">
+        <is>
+          <t>https://huckberry.com/store/flint-and-tinder/category/p/71015-flannel-lined-waxed-trucker-jacket</t>
+        </is>
+      </c>
+      <c r="J6" s="8" t="inlineStr">
+        <is>
+          <t>Dual-flap denser options (Quince/Gap/Blakely) stay on Add-ons as backups</t>
         </is>
       </c>
     </row>
@@ -1389,7 +1389,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:J20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1502,57 +1502,57 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>TOP if shanks OK</t>
+          <t>Alt — best dual flaps + color if shanks OK</t>
         </is>
       </c>
     </row>
     <row r="3" ht="48" customHeight="1">
-      <c r="A3" s="2" t="n">
+      <c r="A3" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>Flint &amp; Tinder Flannel-Lined Waxed Trucker (Huckberry)</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="8" t="inlineStr">
         <is>
           <t>Forest</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" s="8" t="inlineStr">
         <is>
           <t>Martexin 7oz waxed sailcloth; USA</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" s="8" t="inlineStr">
         <is>
           <t>Antique-finish metal (matte-er)</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F3" s="8" t="inlineStr">
         <is>
           <t>$328</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="G3" s="8" t="inlineStr">
         <is>
           <t>LIVE — L~389 XL~178</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="H3" s="9" t="inlineStr">
         <is>
           <t>https://huckberry.com/store/flint-and-tinder/category/p/71015-flannel-lined-waxed-trucker-jacket</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="I3" s="8" t="inlineStr">
         <is>
           <t>Great color; only ONE chest flap</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>TOP if matte hardware &gt; dual flaps</t>
+      <c r="J3" s="8" t="inlineStr">
+        <is>
+          <t>LOCKED — Lyle: closest so far (2026-09-05)</t>
         </is>
       </c>
     </row>
@@ -1856,6 +1856,17 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
+    <row r="11"/>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId1"/>
@@ -1875,7 +1886,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -1972,6 +1983,13 @@
         </is>
       </c>
     </row>
+    <row r="14" ht="40" customHeight="1">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-05: Lyle locked Slot 5 = Flint &amp; Tinder Forest waxed trucker $328 (Huckberry). Closest match so far; single chest flap accepted vs dual-flap alts.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>